<commit_message>
Updated location url for azmld location to open VWO test A.
</commit_message>
<xml_diff>
--- a/Data/locationsv2.xlsx
+++ b/Data/locationsv2.xlsx
@@ -73,14 +73,7 @@
     <t>Run GS for azmld</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>https://development.altogetherfuneral.com/funeral-cremation/arizona/mesa/meldrum-mortuary-crematory/azmld.html</t>
-    </r>
+    <t>https://development.altogetherfuneral.com/funeral-cremation/arizona/mesa/meldrum-mortuary-crematory/azmld.html?cac&amp;_vis_preview_data=eyJhIjoiYTE1MTUyYWNhY2I2MTU2ZDJlZWQxNzRlZmFkYjhmMWMiLCJlIjp7IjEzNSI6eyJ2IjoiMSIsImQiOjAsInMiOjAsInRnIjowLCJ0IjowLCJ0ZCI6MCwibCI6MCwiYWxoIjowLCJpcGxlIjowLCJpaG8iOjAsInBhaGkiOm51bGwsInNhYmVyIjpudWxsLCJuZXdRdWVyeUJveCI6bnVsbCwiZGF0YVJlZ2lvbiI6bnVsbCwibWF0Y2hUeXBlIjpudWxsLCJjbiI6InVuZGVmaW5lZCIsInVybCI6Imh0dHBzJTI1M0ElMjUyRiUyNTJGZGV2ZWxvcG1lbnQuYWx0b2dldGhlcmZ1bmVyYWwuY29tJTI1MkZmdW5lcmFsLWNyZW1hdGlvbiUyNTJGYXJpem9uYSUyNTJGbW9oYXZlLXZhbGxleSUyNTJGZGVzZXJ0LWxhd24tZnVuZXJhbC1ob21lLW1vaGF2ZSUyNTJGYXpzZG0uaHRtbCIsImFwcCI6ImFwcCIsInRzIjoxNzYwNTA1NTY4ODM0fX19</t>
   </si>
   <si>
     <t>azmld</t>
@@ -1002,7 +995,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1022,6 +1015,10 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1037,7 +1034,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1052,6 +1049,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1318,7 +1318,7 @@
       <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="3" t="s">

</xml_diff>